<commit_message>
chore(cq-mobile): sync app - readiness report, and the two fixes the fact-check found
A verification pass over the readiness document found a live App Store
2.1 defect (an ungated Google button on the registration screen) and that
the failed-refresh fix had covered two of eight screens. Both closed.

The report and DATA_SAFETY.md are rewritten against recomputed figures and
now carry three launch blockers the first draft omitted: email does not
send, Elasticsearch needs provisioning separately, and object storage is
unconfigured.

Suite 436, analyzer clean. Only cq-mobile/ is touched.
</commit_message>
<xml_diff>
--- a/cq-mobile/docs/TRACKER.xlsx
+++ b/cq-mobile/docs/TRACKER.xlsx
@@ -659,7 +659,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CQ-007</t>
+          <t>CQ-005</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Login, registration and password reset have zero test coverage</t>
+          <t>No prepared inputs for Play Data Safety, Apple privacy labels, or the content-rating questionnaire</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmed. `grep -l auth_repository test/*.dart` returns only test/session_probe_test.dart, and every call in that file is `repo.probeSession()` — login(), register() and the 3-step OTP reset are exercised by nothing. `_userFrom` and the status→message map are exactly where the auditor said. Severity downgraded from ship-blocker to important: I cross-checked the envelope against the live backend and `apps/api/src/auth/auth.controller.ts:147` returns `{ user: publicUser(result.user) }`, which is precisely what `_userFrom` parses, so the catastrophic scenario the auditor invoked ('if the server </t>
+          <t>Prepared 20 Aug in docs/DATA_SAFETY.md, read out of the code with the file behind every claim. Four inputs still block submission and none are app work: a published privacy policy URL, a web deletion URL, retention periods, and whether sending a profile to a recruiter is declared as sharing.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CQ-008</t>
+          <t>CQ-007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>The apply flow's error branches are untested — only its happy-path URL is pinned</t>
+          <t>Login, registration and password reset have zero test coverage</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Confirmed line by line. The apply test at test/jobs_repository_contract_test.dart:80-86 asserts path `/me/applications` and body `{jobId: 7}` and nothing else, and all five error branches in JobsRepository.apply() are unreached by any test — including the quota-vs-throttle discrimination, which really does hinge on a single expression. The interceptor in that same file resolves every request with a 200, so it structurally cannot reach an error branch. Severity trimmed to important on the same basis as the auth finding: the branch logic reads correctly today, so this is uncovered risk rather th</t>
+          <t xml:space="preserve">Confirmed. `grep -l auth_repository test/*.dart` returns only test/session_probe_test.dart, and every call in that file is `repo.probeSession()` — login(), register() and the 3-step OTP reset are exercised by nothing. `_userFrom` and the status→message map are exactly where the auditor said. Severity downgraded from ship-blocker to important: I cross-checked the envelope against the live backend and `apps/api/src/auth/auth.controller.ts:147` returns `{ user: publicUser(result.user) }`, which is precisely what `_userFrom` parses, so the catastrophic scenario the auditor invoked ('if the server </t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CQ-009</t>
+          <t>CQ-008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>The router's auth redirect — the gate between signed-out users and the app — has no test</t>
+          <t>The apply flow's error branches are untested — only its happy-path URL is pinned</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Confirmed. `grep -ln 'app_router' test/*.dart` returns nothing, and app_router.dart does not appear in the full list of package imports across the suite (I dumped `grep -ho 'package:cq_mobile/[^']*' test/*.dart | sort -u` — 29 imports, no core/router). The redirect switch is exactly the three-way gate described. app-independent confirmed and it is genuinely cheap: the redirect is pure logic over a ProviderContainer with authControllerProvider overridden, no device, no network, no account.</t>
+          <t>Confirmed line by line. The apply test at test/jobs_repository_contract_test.dart:80-86 asserts path `/me/applications` and body `{jobId: 7}` and nothing else, and all five error branches in JobsRepository.apply() are unreached by any test — including the quota-vs-throttle discrimination, which really does hinge on a single expression. The interceptor in that same file resolves every request with a 200, so it structurally cannot reach an error branch. Severity trimmed to important on the same basis as the auth finding: the branch logic reads correctly today, so this is uncovered risk rather th</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CQ-010</t>
+          <t>CQ-009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>JobFilters — all of search filtering and the alert built from it — is completely untested</t>
+          <t>The router's auth redirect — the gate between signed-out users and the app — has no test</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Confirmed including the subtle part. job_filters.dart is imported by no test. `active` really does compare `x.id != s.id` (lines 116-133) while CatalogItem's `==` is deliberately slug-first with an id-only fallback (catalog_models.dart:37-45), and route-seeded facets really are built with `id: 0` (job_search_screen.dart:96) with the invariant carried only in a comment. test/catalog_item_test.dart pins the slug-first equality but never touches JobFilters.active, so the id-comparison path is untested. The auditor's point about the weak existing assertion is right: test/jobs_repository_contract_t</t>
+          <t>Confirmed. `grep -ln 'app_router' test/*.dart` returns nothing, and app_router.dart does not appear in the full list of package imports across the suite (I dumped `grep -ho 'package:cq_mobile/[^']*' test/*.dart | sort -u` — 29 imports, no core/router). The redirect switch is exactly the three-way gate described. app-independent confirmed and it is genuinely cheap: the redirect is pure logic over a ProviderContainer with authControllerProvider overridden, no device, no network, no account.</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CQ-011</t>
+          <t>CQ-010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>16 of 20 repositories and most response parsers have no test, including account deletion</t>
+          <t>JobFilters — all of search filtering and the alert built from it — is completely untested</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Confirmed by mechanical count with two small corrections. I grepped every repository filename across test/*.dart: 15 return zero hits (alerts, applications, articles, companies, dashboard, education, experience, home, languages, onboarding, profile, projects, saved_jobs, settings, skills) and resume_repository is referenced only by a widget test of the error card — so '16 of 20 with no repository-level test' is accurate. All 16 named model classes return zero hits, parsers_test.dart covers exactly 7 parsers (JobSummary, JobsPage, ApplyQuota, HomeFeed, Application, SavedJob, NotificationPrefere</t>
+          <t>Confirmed including the subtle part. job_filters.dart is imported by no test. `active` really does compare `x.id != s.id` (lines 116-133) while CatalogItem's `==` is deliberately slug-first with an id-only fallback (catalog_models.dart:37-45), and route-seeded facets really are built with `id: 0` (job_search_screen.dart:96) with the invariant carried only in a comment. test/catalog_item_test.dart pins the slug-first equality but never touches JobFilters.active, so the id-comparison path is untested. The auditor's point about the weak existing assertion is right: test/jobs_repository_contract_t</t>
         </is>
       </c>
     </row>
@@ -819,7 +819,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CQ-012</t>
+          <t>CQ-011</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>No integration or e2e test exists, and not one screen is ever mounted in a test</t>
+          <t>16 of 20 repositories and most response parsers have no test, including account deletion</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Confirmed. No integration_test directory, dev_dependencies are only flutter_test/flutter_lints/flutter_launcher_icons/image, and a repo-wide grep for matchesGoldenFile|integration_test|mocktail|mockito|patrol|--coverage|codecov returns nothing outside build artifacts. Five files call pumpWidget and none of the 21 `*_screen.dart` files is imported by any test — I dumped every package import in the suite to check, and no screen appears. Minor correction: 21 screens, not ~26. dependsOn stays app-independent but with a split the owner should hear: widget-level screen tests (mount a screen inside a</t>
+          <t>Confirmed by mechanical count with two small corrections. I grepped every repository filename across test/*.dart: 15 return zero hits (alerts, applications, articles, companies, dashboard, education, experience, home, languages, onboarding, profile, projects, saved_jobs, settings, skills) and resume_repository is referenced only by a widget test of the error card — so '16 of 20 with no repository-level test' is accurate. All 16 named model classes return zero hits, parsers_test.dart covers exactly 7 parsers (JobSummary, JobsPage, ApplyQuota, HomeFeed, Application, SavedJob, NotificationPrefere</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CQ-013</t>
+          <t>CQ-012</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>iPhone landscape and full iPad support are declared but nothing was designed for either</t>
+          <t>No integration or e2e test exists, and not one screen is ever mounted in a test</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Locked to iPhone portrait: Info.plist declares portrait only, the ~ipad orientation key is gone, and TARGETED_DEVICE_FAMILY drops from "1,2" to 1. Android matched with android:screenOrientation="portrait". Apple reviews what the app DECLARES, and this declared a landscape and tablet experience nobody had laid out.</t>
+          <t>Confirmed. No integration_test directory, dev_dependencies are only flutter_test/flutter_lints/flutter_launcher_icons/image, and a repo-wide grep for matchesGoldenFile|integration_test|mocktail|mockito|patrol|--coverage|codecov returns nothing outside build artifacts. Five files call pumpWidget and none of the 21 `*_screen.dart` files is imported by any test — I dumped every package import in the suite to check, and no screen appears. Minor correction: 21 screens, not ~26. dependsOn stays app-independent but with a split the owner should hear: widget-level screen tests (mount a screen inside a</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CQ-014</t>
+          <t>CQ-013</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Registration collects a marketing-consent checkbox and throws it away</t>
+          <t>iPhone landscape and full iPad support are declared but nothing was designed for either</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Unticking now PATCHes /me/notifications (alerts + product news off). Copy no longer promises SMS.</t>
+          <t>Locked to iPhone portrait: Info.plist declares portrait only, the ~ipad orientation key is gone, and TARGETED_DEVICE_FAMILY drops from "1,2" to 1. Android matched with android:screenOrientation="portrait". Apple reviews what the app DECLARES, and this declared a landscape and tablet experience nobody had laid out.</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CQ-015</t>
+          <t>CQ-014</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Sharing a company sends a link the website 404s</t>
+          <t>Registration collects a marketing-consent checkbox and throws it away</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Was my own regression from earlier the same night. Now emits &lt;slug&gt;-overview-&lt;id&gt; per buildCompanyHandle.</t>
+          <t>Unticking now PATCHes /me/notifications (alerts + product news off). Copy no longer promises SMS.</t>
         </is>
       </c>
     </row>
@@ -947,7 +947,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CQ-016</t>
+          <t>CQ-015</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Every server-side validation error shows as "Something went wrong. Please try again."</t>
+          <t>Sharing a company sends a link the website 404s</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>friendlyDioMessage now reads Zod issue arrays and names the field. Root cause of every generic apology in the product.</t>
+          <t>Was my own regression from earlier the same night. Now emits &lt;slug&gt;-overview-&lt;id&gt; per buildCompanyHandle.</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CQ-017</t>
+          <t>CQ-016</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Clearing a text field in the profile or education editor silently does nothing</t>
+          <t>Every server-side validation error shows as "Something went wrong. Please try again."</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Rule extracted to core/format/patch_body.dart with 7 tests. phone stays skipped; preferredCityIds got a _citiesLoaded flag.</t>
+          <t>friendlyDioMessage now reads Zod issue arrays and names the field. Root cause of every generic apology in the product.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CQ-018</t>
+          <t>CQ-017</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Tapping "Next page" produces no visible response and leaves the user parked at the bottom of the list</t>
+          <t>Clearing a text field in the profile or education editor silently does nothing</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Only pull-to-refresh keeps the list mounted now; the pager, a new query and filter changes show the loader and rebuild at the top.</t>
+          <t>Rule extracted to core/format/patch_body.dart with 7 tests. phone stays skipped; preferredCityIds got a _citiesLoaded flag.</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CQ-019</t>
+          <t>CQ-018</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>The Jobs tab never refreshes its saved/applied markers after the user saves or applies</t>
+          <t>Tapping "Next page" produces no visible response and leaves the user parked at the bottom of the list</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Listens on CqData and refetches just the markers. Also fixed _enrichMarkers bailing on an empty reply.</t>
+          <t>Only pull-to-refresh keeps the list mounted now; the pager, a new query and filter changes show the loader and rebuild at the top.</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CQ-020</t>
+          <t>CQ-019</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Profile's Resume card still says "Add your resume to apply for jobs" after the user uploads one during the apply flow</t>
+          <t>The Jobs tab never refreshes its saved/applied markers after the user saves or applies</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Added CqData.resume, bumped from the single upload funnel, so profile/apply/onboarding all agree.</t>
+          <t>Listens on CqData and refetches just the markers. Also fixed _enrichMarkers bailing on an empty reply.</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CQ-021</t>
+          <t>CQ-020</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>"Continue with Phone" and "Log in with OTP" are finished-looking dead ends</t>
+          <t>Profile's Resume card still says "Add your resume to apply for jobs" after the user uploads one during the apply flow</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Covered by the same AppConfig.showAuthAlternatives gate.</t>
+          <t>Added CqData.resume, bumped from the single upload funnel, so profile/apply/onboarding all agree.</t>
         </is>
       </c>
     </row>
@@ -1139,17 +1139,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CQ-022</t>
+          <t>CQ-021</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Debug Dio logger prints auth request bodies — plaintext password, OTP code and reset ticket reach logcat</t>
+          <t>"Continue with Phone" and "Log in with OTP" are finished-looking dead ends</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Replaced LogInterceptor with a redacting one. 7 tests, mutation-checked.</t>
+          <t>Covered by the same AppConfig.showAuthAlternatives gate.</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CQ-024</t>
+          <t>CQ-022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>ITSAppUsesNonExemptEncryption is not declared — every iOS upload will stall on the export-compliance prompt</t>
+          <t>Debug Dio logger prints auth request bodies — plaintext password, OTP code and reset ticket reach logcat</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Duplicate of the P1 row filed by another auditor; declared false in the same pass.</t>
+          <t>Replaced LogInterceptor with a redacting one. 7 tests, mutation-checked.</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CQ-025</t>
+          <t>CQ-024</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>No coverage is measured anywhere, so "155 tests" has no denominator</t>
+          <t>ITSAppUsesNonExemptEncryption is not declared — every iOS upload will stall on the export-compliance prompt</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>CI runs --coverage, summarises with lcov, uploads lcov.info.</t>
+          <t>Duplicate of the P1 row filed by another auditor; declared false in the same pass.</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CQ-026</t>
+          <t>CQ-025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>CI has no formatting gate and floats its Flutter version while failing on any analyzer output</t>
+          <t>No coverage is measured anywhere, so "155 tests" has no denominator</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Flutter pinned to 3.41.0; coverage added. Format gate deliberately deferred - 117 of 155 files are unformatted, so it belongs in its own reviewed commit.</t>
+          <t>CI runs --coverage, summarises with lcov, uploads lcov.info.</t>
         </is>
       </c>
     </row>
@@ -1267,7 +1267,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CQ-027</t>
+          <t>CQ-026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>No Android App Bundle has ever been built; the only release pipeline produces an APK</t>
+          <t>CI has no formatting gate and floats its Flutter version while failing on any analyzer output</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>CI release step now builds an .aab with production URLs. Not runnable locally until the Gradle fault clears.</t>
+          <t>Flutter pinned to 3.41.0; coverage added. Format gate deliberately deferred - 117 of 155 files are unformatted, so it belongs in its own reviewed commit.</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CQ-028</t>
+          <t>CQ-027</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Nothing fails a release build that still has the localhost API default baked in</t>
+          <t>No Android App Bundle has ever been built; the only release pipeline produces an APK</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>AppConfig.pointsAtLocalhost + assert + release_config_test.dart.</t>
+          <t>CI release step now builds an .aab with production URLs. Not runnable locally until the Gradle fault clears.</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CQ-031</t>
+          <t>CQ-028</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>The hand-off spec in the app repo still tells the next developer the endpoints have no /v1 prefix</t>
+          <t>Nothing fails a release build that still has the localhost API default baked in</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>API_SPEC_FOR_MOBILE.md said "no global route prefix". The truth is a SPLIT surface: main.ts sets defaultVersion VERSION_NEUTRAL, so /v1 applies only where a controller asks for it — the public surface does, /me/* and auth/* do not. Corrected with both sides spelled out, because a route added on the wrong side 404s in a way nothing in CI would catch.</t>
+          <t>AppConfig.pointsAtLocalhost + assert + release_config_test.dart.</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CQ-032</t>
+          <t>CQ-031</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Creating or deleting an alert from the Alerts screen leaves Home's alert count wrong</t>
+          <t>The hand-off spec in the app repo still tells the next developer the endpoints have no /v1 prefix</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Alerts screen now bumps the freshness bus, so Home stops showing a stale count.</t>
+          <t>API_SPEC_FOR_MOBILE.md said "no global route prefix". The truth is a SPLIT surface: main.ts sets defaultVersion VERSION_NEUTRAL, so /v1 applies only where a controller asks for it — the public surface does, /me/* and auth/* do not. Corrected with both sides spelled out, because a route added on the wrong side 404s in a way nothing in CI would catch.</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1395,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CQ-033</t>
+          <t>CQ-032</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Remaining places that invent a value instead of admitting it is unknown</t>
+          <t>Creating or deleting an alert from the Alerts screen leaves Home's alert count wrong</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>savedAt/appliedAt/updatedAt/at nullable; resume uploadedAt no longer claims "Added today".</t>
+          <t>Alerts screen now bumps the freshness bus, so Home stops showing a stale count.</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CQ-034</t>
+          <t>CQ-033</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Job detail replaces a job that loaded fine with "Could not load this job" if a secondary call throws</t>
+          <t>Remaining places that invent a value instead of admitting it is unknown</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Each enrichment call has its own catch; only the job itself can error the screen.</t>
+          <t>savedAt/appliedAt/updatedAt/at nullable; resume uploadedAt no longer claims "Added today".</t>
         </is>
       </c>
     </row>
@@ -1459,123 +1459,123 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t>CQ-034</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Job detail replaces a job that loaded fine with "Could not load this job" if a secondary call throws</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>nothing - can be done now</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Each enrichment call has its own catch; only the job itself can error the screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>CQ-035</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>Undisposed TextEditingController in the delete-account dialog</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>nothing - can be done now</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>nothing - can be done now</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Disposed after the delete-account dialog closes.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>CQ-006</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>CI cannot run from the snapshot branch (the code itself is now pushed and current)</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>nothing - can be done now</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>nothing - can be done now</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>Resolved in part on 20 Aug: the jobportal app/cq-mobile branch now carries the full app, all 435 tests and the workflow file. What remains is structural — GitHub Actions only reads .github/workflows/ at the ROOT of a repository, and the app lives under cq-mobile/ there, so ci.yml still cannot run. Fixing it needs either a repo of its own for the app, or a root-level workflow on the shared repo, which would be that repo’s first and needs the website owner’s agreement.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Not doing</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>CQ-023</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>No screenshot/recents protection (FLAG_SECURE) on profile, resume or application screens</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>nothing - can be done now</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>nothing - can be done now</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Deliberately NOT doing this. FLAG_SECURE blanks the app in the recents switcher and blocks screenshots wholesale — which breaks a candidate screenshotting their own application status or resume to share, a thing people genuinely do. The data here is the user's own CV and job history, not credentials or payment details. Revisit only if a customer or a review asks for it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>CQ-005</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>No prepared inputs for Play Data Safety, Apple privacy labels, or the content-rating questionnaire</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>nothing - can be done now</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>CONFIRMED as a real gap, but I am CORRECTING the classification from 'owner' to 'app-independent'. The deliverable named here is prepared INPUTS — a written inventory mapping each collected field to its Play Data Safety category and Apple nutrition-label bucket, plus draft answers to the UGC/age questions. That inventory is derived entirely from code the app dev already owns (candidate_profile.dart, resume_section.dart, the Dio repositories) and can be written tonight on Windows with no keystore, URL, account or endpoint. Only the final keystroke — entering it into the two Consoles — needs the</t>
         </is>
       </c>
     </row>
@@ -2138,14 +2138,14 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CQ-051</t>
+          <t>CQ-052</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>No privacy policy or terms page exists on the website — the URL both Consoles require as a mandatory field has no destination</t>
+          <t>Play Data Safety requires a web-based account/data-deletion URL in addition to the in-app path</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2165,7 +2165,7 @@
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>CONFIRMED with my own greps, including the two escape hatches the original auditor did not check — the Next 16 catch-all route and the site footer. Neither provides a legal page. dependsOn=website is correct: the deliverable is a route on apps/web that only the web dev can add; the owner supplies the policy text but has nothing to supply it into. Not app-independent under any reading.</t>
+          <t>Prepared 20 Aug in docs/DATA_SAFETY.md, read out of the code with the file behind every claim. Four inputs still block submission and none are app work: a published privacy policy URL, a web deletion URL, retention periods, and whether sending a profile to a recruiter is declared as sharing.</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CQ-052</t>
+          <t>CQ-051</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>Play Data Safety requires a web-based account/data-deletion URL in addition to the in-app path</t>
+          <t>No privacy policy or terms page exists on the website — the URL both Consoles require as a mandatory field has no destination</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>CONFIRMED. I specifically tried to refute this by proving the in-app path was incomplete — it is not, it is fully wired including the disabled-button state and post-delete logout, so the auditor was right to credit it. What remains is only the Play Console 'Data deletion' web URL, which Play requires for any app supporting in-app account creation and which no route on apps/web serves. dependsOn=website is correct — a hosted request page is not something the app dev can produce.</t>
+          <t>CONFIRMED with my own greps, including the two escape hatches the original auditor did not check — the Next 16 catch-all route and the site footer. Neither provides a legal page. dependsOn=website is correct: the deliverable is a route on apps/web that only the web dev can add; the owner supplies the policy text but has nothing to supply it into. Not app-independent under any reading.</t>
         </is>
       </c>
     </row>

</xml_diff>